<commit_message>
Update: changed date format
</commit_message>
<xml_diff>
--- a/qlb_colony_spreadsheet.xlsx
+++ b/qlb_colony_spreadsheet.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sheinasim/Bioinformatic_software/sheinasim.github.io/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usdagcc-my.sharepoint.com/personal/sheina_sim_usda_gov/Documents/Projects/Dashboard/sheinasim.github.io/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E79CA08-09BD-E04C-8D25-9DEEB81A32E7}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{3E79CA08-09BD-E04C-8D25-9DEEB81A32E7}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{8910B4DB-A138-D34C-99A7-2FA921AB4154}"/>
   <bookViews>
-    <workbookView xWindow="-29000" yWindow="4300" windowWidth="29020" windowHeight="9940" xr2:uid="{B6248D05-47C7-5D4A-B216-529F4D1EBA26}"/>
+    <workbookView xWindow="-32720" yWindow="60" windowWidth="29020" windowHeight="9940" xr2:uid="{B6248D05-47C7-5D4A-B216-529F4D1EBA26}"/>
   </bookViews>
   <sheets>
     <sheet name="lifestages" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
     <t>Adult male</t>
   </si>
   <si>
-    <t>2021March12</t>
+    <t>2021.03.12</t>
   </si>
 </sst>
 </file>

</xml_diff>